<commit_message>
add reports Official Housing week
</commit_message>
<xml_diff>
--- a/Data Audit/الافرع قبل التصميم.xlsx
+++ b/Data Audit/الافرع قبل التصميم.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Projects\reports\Data Audit\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0256FC85-7805-4B7C-9BAD-3F8EE1918A65}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FD39EFE9-78AB-468D-8E3A-DE460870B931}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="29" uniqueCount="21">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="27" uniqueCount="20">
   <si>
     <t>أرشفة البريد إلكترونياً وورقياً</t>
   </si>
@@ -71,9 +71,6 @@
   </si>
   <si>
     <t>إعداد مذكرات عرض للسيد الوزير (  تعديل مسمى وظيفي )</t>
-  </si>
-  <si>
-    <t>35%</t>
   </si>
   <si>
     <t>100%</t>
@@ -227,7 +224,7 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -253,6 +250,7 @@
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="3"/>
+    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="4">
     <cellStyle name="عادي" xfId="0" builtinId="0"/>
@@ -546,50 +544,50 @@
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A1" s="10" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="B1" s="10" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A2" s="10" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="B2" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A3" s="10" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="B3" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A4" s="10" t="s">
-        <v>14</v>
-      </c>
-      <c r="B4" t="s">
-        <v>12</v>
+        <v>13</v>
+      </c>
+      <c r="B4" s="11">
+        <v>0.55000000000000004</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A5" s="10" t="s">
-        <v>19</v>
-      </c>
-      <c r="B5" t="s">
-        <v>11</v>
+        <v>18</v>
+      </c>
+      <c r="B5" s="11">
+        <v>0.53</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A6" s="10" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B6" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
     </row>
   </sheetData>
@@ -609,10 +607,10 @@
   <sheetData>
     <row r="1" spans="1:2" ht="15" x14ac:dyDescent="0.2">
       <c r="A1" s="10" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="B1" s="10" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.2">
@@ -710,10 +708,10 @@
   <sheetData>
     <row r="1" spans="1:15" ht="26.25" x14ac:dyDescent="0.2">
       <c r="A1" s="10" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="B1" s="10" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="C1" s="9"/>
       <c r="D1" s="9"/>
@@ -815,7 +813,7 @@
     </row>
     <row r="6" spans="1:15" ht="25.15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A6" s="6" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="B6" s="5">
         <v>5</v>

</xml_diff>